<commit_message>
Ship upgraded Budget-Based Diet Maker snapshot
Publish the latest improved project iteration with the current working app state and add a comprehensive README for setup, architecture, and API usage.
</commit_message>
<xml_diff>
--- a/backend/Userinfo.xlsx
+++ b/backend/Userinfo.xlsx
@@ -831,7 +831,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H36"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -855,6 +855,9 @@
       <c r="G1" t="str">
         <v>budget</v>
       </c>
+      <c r="H1" t="str">
+        <v>preference</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1224,9 +1227,485 @@
         <v>2000</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B18" t="str">
+        <v>25</v>
+      </c>
+      <c r="C18" t="str">
+        <v>178</v>
+      </c>
+      <c r="D18" t="str">
+        <v>65</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G18" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B19" t="str">
+        <v>25</v>
+      </c>
+      <c r="C19" t="str">
+        <v>178</v>
+      </c>
+      <c r="D19" t="str">
+        <v>65</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Weight Loss</v>
+      </c>
+      <c r="G19" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>aki</v>
+      </c>
+      <c r="B20" t="str">
+        <v>34</v>
+      </c>
+      <c r="C20" t="str">
+        <v>176</v>
+      </c>
+      <c r="D20" t="str">
+        <v>67</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Weight Loss</v>
+      </c>
+      <c r="G20" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B21" t="str">
+        <v>25</v>
+      </c>
+      <c r="C21" t="str">
+        <v>178</v>
+      </c>
+      <c r="D21" t="str">
+        <v>65</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G21" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B22" t="str">
+        <v>25</v>
+      </c>
+      <c r="C22" t="str">
+        <v>178</v>
+      </c>
+      <c r="D22" t="str">
+        <v>65</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G22" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B23" t="str">
+        <v>25</v>
+      </c>
+      <c r="C23" t="str">
+        <v>178</v>
+      </c>
+      <c r="D23" t="str">
+        <v>65</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G23" t="str">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B24" t="str">
+        <v>25</v>
+      </c>
+      <c r="C24" t="str">
+        <v>178</v>
+      </c>
+      <c r="D24" t="str">
+        <v>65</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Weight Loss</v>
+      </c>
+      <c r="G24" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H24" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B25" t="str">
+        <v>25</v>
+      </c>
+      <c r="C25" t="str">
+        <v>178</v>
+      </c>
+      <c r="D25" t="str">
+        <v>65</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G25" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H25" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B26" t="str">
+        <v>25</v>
+      </c>
+      <c r="C26" t="str">
+        <v>178</v>
+      </c>
+      <c r="D26" t="str">
+        <v>65</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G26" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H26" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B27" t="str">
+        <v>25</v>
+      </c>
+      <c r="C27" t="str">
+        <v>178</v>
+      </c>
+      <c r="D27" t="str">
+        <v>65</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G27" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H27" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B28" t="str">
+        <v>25</v>
+      </c>
+      <c r="C28" t="str">
+        <v>178</v>
+      </c>
+      <c r="D28" t="str">
+        <v>65</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G28" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H28" t="str">
+        <v>non-veg</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B29" t="str">
+        <v>25</v>
+      </c>
+      <c r="C29" t="str">
+        <v>178</v>
+      </c>
+      <c r="D29" t="str">
+        <v>65</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G29" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H29" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B30" t="str">
+        <v>25</v>
+      </c>
+      <c r="C30" t="str">
+        <v>178</v>
+      </c>
+      <c r="D30" t="str">
+        <v>65</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G30" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H30" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B31" t="str">
+        <v>25</v>
+      </c>
+      <c r="C31" t="str">
+        <v>178</v>
+      </c>
+      <c r="D31" t="str">
+        <v>65</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G31" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H31" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B32" t="str">
+        <v>25</v>
+      </c>
+      <c r="C32" t="str">
+        <v>178</v>
+      </c>
+      <c r="D32" t="str">
+        <v>65</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G32" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H32" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B33" t="str">
+        <v>25</v>
+      </c>
+      <c r="C33" t="str">
+        <v>178</v>
+      </c>
+      <c r="D33" t="str">
+        <v>65</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G33" t="str">
+        <v>2000</v>
+      </c>
+      <c r="H33" t="str">
+        <v>non-veg</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B34" t="str">
+        <v>25</v>
+      </c>
+      <c r="C34" t="str">
+        <v>178</v>
+      </c>
+      <c r="D34" t="str">
+        <v>65</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Weight Maintenance</v>
+      </c>
+      <c r="G34" t="str">
+        <v>500</v>
+      </c>
+      <c r="H34" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B35" t="str">
+        <v>25</v>
+      </c>
+      <c r="C35" t="str">
+        <v>178</v>
+      </c>
+      <c r="D35" t="str">
+        <v>65</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G35" t="str">
+        <v>500</v>
+      </c>
+      <c r="H35" t="str">
+        <v>veg</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>akilesh</v>
+      </c>
+      <c r="B36" t="str">
+        <v>25</v>
+      </c>
+      <c r="C36" t="str">
+        <v>178</v>
+      </c>
+      <c r="D36" t="str">
+        <v>65</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Male</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Weight Gain</v>
+      </c>
+      <c r="G36" t="str">
+        <v>500</v>
+      </c>
+      <c r="H36" t="str">
+        <v>veg</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H36"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>